<commit_message>
feat: PushMap pathing polish, GoalKind debug labels, SoftCollision B+ SPEC
Tighten spawn leash/advance hold/kill reach; add soldier GoalKind debug labels; draft SoftCollision CombatMoveMode slices and SPEC.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Gravedigger2026/Assets/ConfigTables/Excel/推图战_推图战配置表_PushMap_PushMapGameplayConfig.xlsx
+++ b/Gravedigger2026/Assets/ConfigTables/Excel/推图战_推图战配置表_PushMap_PushMapGameplayConfig.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t>玩法配置ID</t>
   </si>
@@ -122,9 +122,6 @@
   </si>
   <si>
     <t>Dungeon_Stub_01</t>
-  </si>
-  <si>
-    <t>5</t>
   </si>
   <si>
     <t>PM-02 sample</t>
@@ -140,14 +137,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="21">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -609,148 +599,148 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1210,11 +1200,11 @@
       <c r="F4" t="s">
         <v>29</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4">
+        <v>2</v>
+      </c>
+      <c r="H4" t="s">
         <v>30</v>
-      </c>
-      <c r="H4" t="s">
-        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>